<commit_message>
Update daily screener results
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -22735,8 +22735,8 @@
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="T1:U1"/>
+    <mergeCell ref="V1:W1"/>
     <mergeCell ref="K1:L1"/>
-    <mergeCell ref="V1:W1"/>
     <mergeCell ref="X1:Y1"/>
     <mergeCell ref="Z1:AA1"/>
     <mergeCell ref="O1:P1"/>
@@ -23091,7 +23091,7 @@
         <v>2</v>
       </c>
       <c r="D4" s="305" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4" s="306" t="n">
         <v>243.11</v>
@@ -23180,7 +23180,7 @@
         <v>3</v>
       </c>
       <c r="D5" s="305" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" s="306" t="n">
         <v>214.56</v>
@@ -23257,264 +23257,264 @@
     <row r="6" ht="17" customHeight="1" s="203">
       <c r="A6" s="303" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>U</t>
         </is>
       </c>
       <c r="B6" s="304" t="inlineStr">
         <is>
-          <t>Block, Inc</t>
+          <t>Unity Soft</t>
         </is>
       </c>
       <c r="C6" s="305" t="n">
         <v>4</v>
       </c>
       <c r="D6" s="305" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E6" s="306" t="n">
-        <v>77.3</v>
+        <v>30.89</v>
       </c>
       <c r="F6" s="307" t="n">
-        <v>-1.94</v>
+        <v>5.35</v>
       </c>
       <c r="G6" s="306" t="n">
-        <v>81.11</v>
+        <v>49.47</v>
       </c>
       <c r="H6" s="308" t="n">
-        <v>275</v>
+        <v>213</v>
       </c>
       <c r="I6" s="306" t="n">
-        <v>81.11</v>
+        <v>49.47</v>
       </c>
       <c r="J6" s="308" t="n">
-        <v>275</v>
-      </c>
-      <c r="K6" s="309" t="n"/>
-      <c r="L6" s="308" t="n"/>
+        <v>213</v>
+      </c>
+      <c r="K6" s="309" t="n">
+        <v>46051</v>
+      </c>
+      <c r="L6" s="308" t="n">
+        <v>162</v>
+      </c>
       <c r="M6" s="310" t="n">
-        <v>1.962992338452117</v>
+        <v>2.287752253146536</v>
       </c>
       <c r="N6" s="307" t="n">
-        <v>0.14</v>
+        <v>1.3</v>
       </c>
       <c r="O6" s="310" t="n">
-        <v>56.63701812217888</v>
+        <v>62.9270295393946</v>
       </c>
       <c r="P6" s="307" t="n">
-        <v>-7.56</v>
+        <v>11.19</v>
       </c>
       <c r="Q6" s="311" t="n">
-        <v>3.72</v>
+        <v>5.39</v>
       </c>
       <c r="R6" s="312" t="n">
-        <v>1.721026215962425</v>
+        <v>0.7269090842337533</v>
       </c>
       <c r="S6" s="307" t="n">
-        <v>-8.119999999999999</v>
+        <v>93.98</v>
       </c>
       <c r="T6" s="312" t="n">
-        <v>1.581901707324438</v>
+        <v>0.4414177593734833</v>
       </c>
       <c r="U6" s="307" t="n">
-        <v>27.17</v>
+        <v>78.58</v>
       </c>
       <c r="V6" s="312" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.65</t>
         </is>
       </c>
       <c r="W6" s="307" t="n">
-        <v>1.087947631634646</v>
+        <v>1.646759942929066</v>
       </c>
       <c r="X6" s="313" t="n">
-        <v>461714055.1857258</v>
+        <v>361150003.4183065</v>
       </c>
       <c r="Y6" s="307" t="n">
-        <v>-0.79</v>
+        <v>-0.26</v>
       </c>
       <c r="Z6" s="309" t="n">
         <v>46149</v>
       </c>
       <c r="AA6" s="314" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
     </row>
     <row r="7" ht="17" customHeight="1" s="203">
       <c r="A7" s="303" t="inlineStr">
         <is>
-          <t>U</t>
+          <t>BABA</t>
         </is>
       </c>
       <c r="B7" s="304" t="inlineStr">
         <is>
-          <t>Unity Soft</t>
+          <t>Alibaba Gr</t>
         </is>
       </c>
       <c r="C7" s="305" t="n">
         <v>5</v>
       </c>
       <c r="D7" s="305" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" s="306" t="n">
-        <v>30.89</v>
+        <v>112.33</v>
       </c>
       <c r="F7" s="307" t="n">
-        <v>5.35</v>
+        <v>16.84</v>
       </c>
       <c r="G7" s="306" t="n">
-        <v>49.47</v>
+        <v>189.34</v>
       </c>
       <c r="H7" s="308" t="n">
-        <v>213</v>
+        <v>281</v>
       </c>
       <c r="I7" s="306" t="n">
-        <v>49.47</v>
+        <v>189.34</v>
       </c>
       <c r="J7" s="308" t="n">
-        <v>213</v>
+        <v>281</v>
       </c>
       <c r="K7" s="309" t="n">
-        <v>46051</v>
+        <v>46182</v>
       </c>
       <c r="L7" s="308" t="n">
-        <v>162</v>
+        <v>31</v>
       </c>
       <c r="M7" s="310" t="n">
-        <v>2.287752253146536</v>
+        <v>1.258054502290484</v>
       </c>
       <c r="N7" s="307" t="n">
-        <v>1.3</v>
+        <v>0.75</v>
       </c>
       <c r="O7" s="310" t="n">
-        <v>62.9270295393946</v>
+        <v>55.54302015005555</v>
       </c>
       <c r="P7" s="307" t="n">
-        <v>11.19</v>
+        <v>133.64</v>
       </c>
       <c r="Q7" s="311" t="n">
-        <v>5.39</v>
+        <v>3.57</v>
       </c>
       <c r="R7" s="312" t="n">
-        <v>0.7269090842337533</v>
+        <v>-3.984855606826656</v>
       </c>
       <c r="S7" s="307" t="n">
-        <v>93.98</v>
+        <v>-52.07</v>
       </c>
       <c r="T7" s="312" t="n">
-        <v>0.4414177593734833</v>
+        <v>-6.498684291029949</v>
       </c>
       <c r="U7" s="307" t="n">
-        <v>78.58</v>
+        <v>-11.67</v>
       </c>
       <c r="V7" s="312" t="inlineStr">
         <is>
-          <t>1.65</t>
+          <t>0.61</t>
         </is>
       </c>
       <c r="W7" s="307" t="n">
-        <v>1.646759942929066</v>
+        <v>0.6131788264167412</v>
       </c>
       <c r="X7" s="313" t="n">
-        <v>361150003.4183065</v>
+        <v>1637003528.623064</v>
       </c>
       <c r="Y7" s="307" t="n">
-        <v>-0.26</v>
+        <v>-1.16</v>
       </c>
       <c r="Z7" s="309" t="n">
-        <v>46149</v>
+        <v>46155</v>
       </c>
       <c r="AA7" s="314" t="n">
-        <v>46240</v>
+        <v>46269</v>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1" s="203">
       <c r="A8" s="303" t="inlineStr">
         <is>
-          <t>BABA</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="B8" s="304" t="inlineStr">
         <is>
-          <t>Alibaba Gr</t>
+          <t>Block, Inc</t>
         </is>
       </c>
       <c r="C8" s="305" t="n">
         <v>6</v>
       </c>
       <c r="D8" s="305" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E8" s="306" t="n">
-        <v>112.33</v>
+        <v>77.3</v>
       </c>
       <c r="F8" s="307" t="n">
-        <v>16.84</v>
+        <v>-1.94</v>
       </c>
       <c r="G8" s="306" t="n">
-        <v>189.34</v>
+        <v>81.11</v>
       </c>
       <c r="H8" s="308" t="n">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="I8" s="306" t="n">
-        <v>189.34</v>
+        <v>81.11</v>
       </c>
       <c r="J8" s="308" t="n">
-        <v>281</v>
-      </c>
-      <c r="K8" s="309" t="n">
-        <v>46182</v>
-      </c>
-      <c r="L8" s="308" t="n">
-        <v>31</v>
-      </c>
+        <v>275</v>
+      </c>
+      <c r="K8" s="309" t="n"/>
+      <c r="L8" s="308" t="n"/>
       <c r="M8" s="310" t="n">
-        <v>1.258054502290484</v>
+        <v>1.962992338452117</v>
       </c>
       <c r="N8" s="307" t="n">
-        <v>0.75</v>
+        <v>0.14</v>
       </c>
       <c r="O8" s="310" t="n">
-        <v>55.54302015005555</v>
+        <v>56.63701812217888</v>
       </c>
       <c r="P8" s="307" t="n">
-        <v>133.64</v>
+        <v>-7.56</v>
       </c>
       <c r="Q8" s="311" t="n">
-        <v>3.57</v>
+        <v>3.72</v>
       </c>
       <c r="R8" s="312" t="n">
-        <v>-3.984855606826656</v>
+        <v>1.721026215962425</v>
       </c>
       <c r="S8" s="307" t="n">
-        <v>-52.07</v>
+        <v>-8.119999999999999</v>
       </c>
       <c r="T8" s="312" t="n">
-        <v>-6.498684291029949</v>
+        <v>1.581901707324438</v>
       </c>
       <c r="U8" s="307" t="n">
-        <v>-11.67</v>
+        <v>27.17</v>
       </c>
       <c r="V8" s="312" t="inlineStr">
         <is>
-          <t>0.61</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="W8" s="307" t="n">
-        <v>0.6131788264167412</v>
+        <v>1.087947631634646</v>
       </c>
       <c r="X8" s="313" t="n">
-        <v>1637003528.623064</v>
+        <v>461714055.1857258</v>
       </c>
       <c r="Y8" s="307" t="n">
-        <v>-1.16</v>
+        <v>-0.79</v>
       </c>
       <c r="Z8" s="309" t="n">
-        <v>46155</v>
+        <v>46149</v>
       </c>
       <c r="AA8" s="314" t="n">
-        <v>46269</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="9" ht="17" customHeight="1" s="203">
@@ -23532,7 +23532,7 @@
         <v>7</v>
       </c>
       <c r="D9" s="305" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="306" t="n">
         <v>268.4</v>
@@ -23706,7 +23706,7 @@
         <v>9</v>
       </c>
       <c r="D11" s="305" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" s="306" t="n">
         <v>96.94</v>
@@ -23795,7 +23795,7 @@
         <v>10</v>
       </c>
       <c r="D12" s="305" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E12" s="306" t="n">
         <v>13.76</v>
@@ -23882,7 +23882,7 @@
       </c>
       <c r="C13" s="305" t="n"/>
       <c r="D13" s="305" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E13" s="306" t="n">
         <v>47</v>
@@ -23969,7 +23969,7 @@
       </c>
       <c r="C14" s="305" t="n"/>
       <c r="D14" s="305" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="306" t="n">
         <v>225.13</v>
@@ -24056,7 +24056,7 @@
       </c>
       <c r="C15" s="305" t="n"/>
       <c r="D15" s="305" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="306" t="n">
         <v>21.49</v>
@@ -24143,7 +24143,7 @@
       </c>
       <c r="C16" s="305" t="n"/>
       <c r="D16" s="305" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E16" s="306" t="n">
         <v>140.42</v>
@@ -24230,7 +24230,7 @@
       </c>
       <c r="C17" s="305" t="n"/>
       <c r="D17" s="305" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E17" s="306" t="n">
         <v>30.55</v>
@@ -24317,7 +24317,7 @@
       </c>
       <c r="C18" s="305" t="n"/>
       <c r="D18" s="305" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E18" s="306" t="n">
         <v>76.04000000000001</v>
@@ -24404,7 +24404,7 @@
       </c>
       <c r="C19" s="305" t="n"/>
       <c r="D19" s="305" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E19" s="306" t="n">
         <v>143.35</v>
@@ -24491,7 +24491,7 @@
       </c>
       <c r="C20" s="305" t="n"/>
       <c r="D20" s="305" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E20" s="306" t="n">
         <v>55.35</v>
@@ -24578,7 +24578,7 @@
       </c>
       <c r="C21" s="305" t="n"/>
       <c r="D21" s="305" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" s="306" t="n">
         <v>9.359999999999999</v>
@@ -24655,349 +24655,349 @@
     <row r="22" ht="17" customHeight="1" s="203">
       <c r="A22" s="303" t="inlineStr">
         <is>
-          <t>NVO</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B22" s="304" t="inlineStr">
         <is>
-          <t>Novo Nordi</t>
+          <t>Reddit, In</t>
         </is>
       </c>
       <c r="C22" s="305" t="n"/>
       <c r="D22" s="305" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E22" s="306" t="n">
-        <v>49.48</v>
+        <v>195.34</v>
       </c>
       <c r="F22" s="307" t="n">
-        <v>-1.88</v>
+        <v>0.34</v>
       </c>
       <c r="G22" s="306" t="n">
-        <v>71.7</v>
+        <v>270.71</v>
       </c>
       <c r="H22" s="308" t="n">
-        <v>350</v>
+        <v>295</v>
       </c>
       <c r="I22" s="306" t="n">
-        <v>81.05</v>
+        <v>270.71</v>
       </c>
       <c r="J22" s="308" t="n">
-        <v>393</v>
+        <v>295</v>
       </c>
       <c r="K22" s="309" t="n">
-        <v>46055</v>
+        <v>46048</v>
       </c>
       <c r="L22" s="308" t="n">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="M22" s="310" t="n">
-        <v>1.34076365925611</v>
+        <v>1.883107397135316</v>
       </c>
       <c r="N22" s="307" t="n">
-        <v>-0.3</v>
+        <v>0.41</v>
       </c>
       <c r="O22" s="310" t="n">
-        <v>64.49507145549126</v>
+        <v>59.50285661399163</v>
       </c>
       <c r="P22" s="307" t="n">
-        <v>-12.18</v>
+        <v>-4.57</v>
       </c>
       <c r="Q22" s="311" t="n">
-        <v>2.67</v>
+        <v>6.14</v>
       </c>
       <c r="R22" s="312" t="n">
-        <v>1.484220401341943</v>
+        <v>8.748440845886336</v>
       </c>
       <c r="S22" s="307" t="n">
-        <v>-0.55</v>
+        <v>65.78</v>
       </c>
       <c r="T22" s="312" t="n">
-        <v>1.236019108371379</v>
+        <v>6.027191811396905</v>
       </c>
       <c r="U22" s="307" t="n">
-        <v>43.13</v>
+        <v>90.48999999999999</v>
       </c>
       <c r="V22" s="312" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="W22" s="307" t="n">
-        <v>1.200807003135739</v>
+        <v>1.451495343045792</v>
       </c>
       <c r="X22" s="313" t="n">
-        <v>846394277.2563708</v>
+        <v>843279028.0501612</v>
       </c>
       <c r="Y22" s="307" t="n">
-        <v>-4.31</v>
+        <v>-1.03</v>
       </c>
       <c r="Z22" s="309" t="n">
-        <v>46148</v>
+        <v>46142</v>
       </c>
       <c r="AA22" s="314" t="n">
-        <v>46239</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="23" ht="17" customHeight="1" s="203">
       <c r="A23" s="303" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>ARES</t>
         </is>
       </c>
       <c r="B23" s="304" t="inlineStr">
         <is>
-          <t>Reddit, In</t>
+          <t>Ares Manag</t>
         </is>
       </c>
       <c r="C23" s="305" t="n"/>
       <c r="D23" s="305" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23" s="306" t="n">
-        <v>195.34</v>
+        <v>121.81</v>
       </c>
       <c r="F23" s="307" t="n">
-        <v>0.34</v>
+        <v>4.2</v>
       </c>
       <c r="G23" s="306" t="n">
-        <v>270.71</v>
+        <v>192.76</v>
       </c>
       <c r="H23" s="308" t="n">
-        <v>295</v>
+        <v>332</v>
       </c>
       <c r="I23" s="306" t="n">
-        <v>270.71</v>
+        <v>192.76</v>
       </c>
       <c r="J23" s="308" t="n">
-        <v>295</v>
+        <v>332</v>
       </c>
       <c r="K23" s="309" t="n">
-        <v>46048</v>
+        <v>46191</v>
       </c>
       <c r="L23" s="308" t="n">
-        <v>165</v>
+        <v>22</v>
       </c>
       <c r="M23" s="310" t="n">
-        <v>1.883107397135316</v>
+        <v>1.719276344770857</v>
       </c>
       <c r="N23" s="307" t="n">
-        <v>0.41</v>
+        <v>1.59</v>
       </c>
       <c r="O23" s="310" t="n">
-        <v>59.50285661399163</v>
+        <v>51.26980141540249</v>
       </c>
       <c r="P23" s="307" t="n">
-        <v>-4.57</v>
+        <v>14.8</v>
       </c>
       <c r="Q23" s="311" t="n">
-        <v>6.14</v>
+        <v>4.21</v>
       </c>
       <c r="R23" s="312" t="n">
-        <v>8.748440845886336</v>
+        <v>-1.469739067660328</v>
       </c>
       <c r="S23" s="307" t="n">
-        <v>65.78</v>
+        <v>-57</v>
       </c>
       <c r="T23" s="312" t="n">
-        <v>6.027191811396905</v>
+        <v>-1.652351202018689</v>
       </c>
       <c r="U23" s="307" t="n">
-        <v>90.48999999999999</v>
+        <v>45.45</v>
       </c>
       <c r="V23" s="312" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t>0.89</t>
         </is>
       </c>
       <c r="W23" s="307" t="n">
-        <v>1.451495343045792</v>
+        <v>0.8894834620295836</v>
       </c>
       <c r="X23" s="313" t="n">
-        <v>843279028.0501612</v>
+        <v>411361930.2794355</v>
       </c>
       <c r="Y23" s="307" t="n">
-        <v>-1.03</v>
+        <v>-0.51</v>
       </c>
       <c r="Z23" s="309" t="n">
-        <v>46142</v>
+        <v>46143</v>
       </c>
       <c r="AA23" s="314" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
     </row>
     <row r="24" ht="17" customHeight="1" s="203">
       <c r="A24" s="303" t="inlineStr">
         <is>
-          <t>ARES</t>
+          <t>ONON</t>
         </is>
       </c>
       <c r="B24" s="304" t="inlineStr">
         <is>
-          <t>Ares Manag</t>
+          <t>On Holding</t>
         </is>
       </c>
       <c r="C24" s="305" t="n"/>
       <c r="D24" s="305" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" s="306" t="n">
-        <v>121.81</v>
+        <v>38.54</v>
       </c>
       <c r="F24" s="307" t="n">
-        <v>4.2</v>
+        <v>4.64</v>
       </c>
       <c r="G24" s="306" t="n">
-        <v>192.76</v>
+        <v>54.24</v>
       </c>
       <c r="H24" s="308" t="n">
-        <v>332</v>
+        <v>358</v>
       </c>
       <c r="I24" s="306" t="n">
-        <v>192.76</v>
+        <v>60.68</v>
       </c>
       <c r="J24" s="308" t="n">
-        <v>332</v>
+        <v>409</v>
       </c>
       <c r="K24" s="309" t="n">
-        <v>46191</v>
+        <v>46171</v>
       </c>
       <c r="L24" s="308" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="M24" s="310" t="n">
-        <v>1.719276344770857</v>
+        <v>1.417557476683008</v>
       </c>
       <c r="N24" s="307" t="n">
-        <v>1.59</v>
+        <v>-0.33</v>
       </c>
       <c r="O24" s="310" t="n">
-        <v>51.26980141540249</v>
+        <v>57.51727568370867</v>
       </c>
       <c r="P24" s="307" t="n">
-        <v>14.8</v>
+        <v>17.74</v>
       </c>
       <c r="Q24" s="311" t="n">
-        <v>4.21</v>
+        <v>4.14</v>
       </c>
       <c r="R24" s="312" t="n">
-        <v>-1.469739067660328</v>
+        <v>-0.1470206746377229</v>
       </c>
       <c r="S24" s="307" t="n">
-        <v>-57</v>
+        <v>-67.38</v>
       </c>
       <c r="T24" s="312" t="n">
-        <v>-1.652351202018689</v>
+        <v>-0.240385522283252</v>
       </c>
       <c r="U24" s="307" t="n">
-        <v>45.45</v>
+        <v>49.13</v>
       </c>
       <c r="V24" s="312" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.61</t>
         </is>
       </c>
       <c r="W24" s="307" t="n">
-        <v>0.8894834620295836</v>
+        <v>0.6116036990966743</v>
       </c>
       <c r="X24" s="313" t="n">
-        <v>411361930.2794355</v>
+        <v>235218864.5303226</v>
       </c>
       <c r="Y24" s="307" t="n">
-        <v>-0.51</v>
+        <v>-1.46</v>
       </c>
       <c r="Z24" s="309" t="n">
-        <v>46143</v>
+        <v>46154</v>
       </c>
       <c r="AA24" s="314" t="n">
-        <v>46234</v>
+        <v>46245</v>
       </c>
     </row>
     <row r="25" ht="17" customHeight="1" s="203">
       <c r="A25" s="303" t="inlineStr">
         <is>
-          <t>ONON</t>
+          <t>NVO</t>
         </is>
       </c>
       <c r="B25" s="304" t="inlineStr">
         <is>
-          <t>On Holding</t>
+          <t>Novo Nordi</t>
         </is>
       </c>
       <c r="C25" s="305" t="n"/>
       <c r="D25" s="305" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E25" s="306" t="n">
-        <v>38.54</v>
+        <v>49.48</v>
       </c>
       <c r="F25" s="307" t="n">
-        <v>4.64</v>
+        <v>-1.88</v>
       </c>
       <c r="G25" s="306" t="n">
-        <v>54.24</v>
+        <v>71.7</v>
       </c>
       <c r="H25" s="308" t="n">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="I25" s="306" t="n">
-        <v>60.68</v>
+        <v>81.05</v>
       </c>
       <c r="J25" s="308" t="n">
-        <v>409</v>
+        <v>393</v>
       </c>
       <c r="K25" s="309" t="n">
-        <v>46171</v>
+        <v>46055</v>
       </c>
       <c r="L25" s="308" t="n">
-        <v>42</v>
+        <v>158</v>
       </c>
       <c r="M25" s="310" t="n">
-        <v>1.417557476683008</v>
+        <v>1.34076365925611</v>
       </c>
       <c r="N25" s="307" t="n">
-        <v>-0.33</v>
+        <v>-0.3</v>
       </c>
       <c r="O25" s="310" t="n">
-        <v>57.51727568370867</v>
+        <v>64.49507145549126</v>
       </c>
       <c r="P25" s="307" t="n">
-        <v>17.74</v>
+        <v>-12.18</v>
       </c>
       <c r="Q25" s="311" t="n">
-        <v>4.14</v>
+        <v>2.67</v>
       </c>
       <c r="R25" s="312" t="n">
-        <v>-0.1470206746377229</v>
+        <v>1.484220401341943</v>
       </c>
       <c r="S25" s="307" t="n">
-        <v>-67.38</v>
+        <v>-0.55</v>
       </c>
       <c r="T25" s="312" t="n">
-        <v>-0.240385522283252</v>
+        <v>1.236019108371379</v>
       </c>
       <c r="U25" s="307" t="n">
-        <v>49.13</v>
+        <v>43.13</v>
       </c>
       <c r="V25" s="312" t="inlineStr">
         <is>
-          <t>0.61</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="W25" s="307" t="n">
-        <v>0.6116036990966743</v>
+        <v>1.200807003135739</v>
       </c>
       <c r="X25" s="313" t="n">
-        <v>235218864.5303226</v>
+        <v>846394277.2563708</v>
       </c>
       <c r="Y25" s="307" t="n">
-        <v>-1.46</v>
+        <v>-4.31</v>
       </c>
       <c r="Z25" s="309" t="n">
-        <v>46154</v>
+        <v>46148</v>
       </c>
       <c r="AA25" s="314" t="n">
-        <v>46245</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="26" ht="17" customHeight="1" s="203">
@@ -25013,7 +25013,7 @@
       </c>
       <c r="C26" s="305" t="n"/>
       <c r="D26" s="305" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E26" s="306" t="n">
         <v>165.35</v>
@@ -25098,7 +25098,7 @@
       </c>
       <c r="C27" s="305" t="n"/>
       <c r="D27" s="305" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E27" s="306" t="n">
         <v>195</v>
@@ -25174,14 +25174,14 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="X1:Y1"/>
+    <mergeCell ref="V1:W1"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="K1:L1"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="E1:F1"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="T1:U1"/>
-    <mergeCell ref="V1:W1"/>
-    <mergeCell ref="X1:Y1"/>
+    <mergeCell ref="O1:P1"/>
     <mergeCell ref="Z1:AA1"/>
-    <mergeCell ref="O1:P1"/>
     <mergeCell ref="M1:N1"/>
     <mergeCell ref="R1:S1"/>
     <mergeCell ref="I1:J1"/>
@@ -27208,12 +27208,10 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I50" s="207" t="n">
-        <v>46182</v>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I50" s="207" t="n"/>
     </row>
     <row r="51" ht="13.55" customHeight="1" s="203">
       <c r="A51" t="inlineStr">

</xml_diff>